<commit_message>
feat: Oferta katalogowa.bat — launcher UI generatora ofert
</commit_message>
<xml_diff>
--- a/documents/Wzory plików/OFerta katalogowa.xlsx
+++ b/documents/Wzory plików/OFerta katalogowa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arkadiusz\Desktop\Auto-ERP-Agent\documents\Wzory plików\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1BA404F-F7DE-4BB9-B04C-CF8D9E4EB437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F072A2AB-E5FA-42A1-9EA2-C797704FF5C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{45B3745C-1D99-47E5-A00E-76F75396205E}"/>
   </bookViews>
@@ -571,7 +571,7 @@
         <v>11</v>
       </c>
       <c r="D2" s="1">
-        <v>1.1644239601948558</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -585,7 +585,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="1">
-        <v>1.3648099327120504</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -599,7 +599,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="1">
-        <v>1.7748868960259594</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -613,7 +613,7 @@
         <v>14</v>
       </c>
       <c r="D5" s="1">
-        <v>2.2717730795059183</v>
+        <v>2.74</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -627,91 +627,91 @@
         <v>17</v>
       </c>
       <c r="D6" s="1">
-        <v>2.2812287496362389</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D7" s="1">
-        <v>2.6838598446789415</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D8" s="1">
-        <v>3.3627136269471753</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D9" s="1">
-        <v>3.0280049258281783</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D10" s="1">
-        <v>1.3038934466846877</v>
+        <v>1.22</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D11" s="1">
-        <v>1.0129762943363125</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D12" s="1">
-        <v>1.1885430114136635</v>
+        <v>1.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>